<commit_message>
feat(sheets): paint borders, merged cells, fonts and frozen panes
</commit_message>
<xml_diff>
--- a/phase1/sheets-craft/fixtures/formats.xlsx
+++ b/phase1/sheets-craft/fixtures/formats.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="167" formatCode="0;[Red]-0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,10 @@
       <b val="1"/>
       <i val="1"/>
       <color rgb="FFFF0000"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="3">
@@ -49,7 +53,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -57,11 +61,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="FF0000FF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -74,6 +83,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -544,7 +554,374 @@
         <v>3.14159265358979</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Boxed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Merged across two columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Row 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Row 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Row 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Row 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Row 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Row 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Row 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Row 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Row 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Row 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Row 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Row 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Row 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Row 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Row 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Row 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Row 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Row 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Row 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Row 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Row 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Row 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Row 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Row 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Row 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Row 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Row 37</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Row 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Row 39</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Row 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Row 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Row 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Row 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Row 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Row 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Row 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Row 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Row 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Row 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Row 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Row 51</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Row 52</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Row 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Row 54</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Row 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Row 56</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Row 57</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Row 58</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Row 59</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Row 60</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A10:B10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>